<commit_message>
Fix a few layout and component selection issues
- Replace out-of-stock components
- Remove some of the 100nF caps that are in parallel with a larger value
- Swap PTVS3V3 -> SD03
- Swap the PMOS to HSU6119 and the NMOS to DOD130N06 for lower Rds(on)
- Slightly increase the copper area around the FETs
- Reduce the soft-start duration to 47 ms
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -747,7 +747,7 @@
         <v>5</v>
       </c>
       <c r="C2" s="4">
-        <v>27.969999999999999</v>
+        <v>25.629999999999999</v>
       </c>
     </row>
     <row r="3" ht="14.25">
@@ -918,7 +918,7 @@
       </c>
       <c r="B16" s="10"/>
       <c r="C16" s="4">
-        <v>41.969999999999999</v>
+        <v>44.700000000000003</v>
       </c>
       <c r="D16" s="10"/>
     </row>

</xml_diff>

<commit_message>
Thicken walls and add gussets to reduce warping risks
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
     <t>Name</t>
   </si>
@@ -33,7 +33,7 @@
     <t xml:space="preserve">PCB Components</t>
   </si>
   <si>
-    <t xml:space="preserve">Detailed BOM in production/bom.csv</t>
+    <t xml:space="preserve">production/Reflow Plate Controller/BOM-Reflow Plate Controller.csv</t>
   </si>
   <si>
     <t xml:space="preserve">1.3" SSD1315 OLED Display</t>
@@ -123,7 +123,10 @@
     <t xml:space="preserve">JLC3DP (SLS 1172Pro Nylon)</t>
   </si>
   <si>
-    <t xml:space="preserve">JLC Shipping</t>
+    <t xml:space="preserve">JLCPCB Shipping</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JLC3DP Shipping</t>
   </si>
   <si>
     <t xml:space="preserve">LCSC Shipping</t>
@@ -180,7 +183,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -196,6 +199,7 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
       <protection hidden="0" locked="1"/>
@@ -722,7 +726,7 @@
     <col customWidth="1" min="1" max="1" width="29.28125"/>
     <col customWidth="1" min="2" max="2" width="29.421875"/>
     <col customWidth="1" min="3" max="3" width="12.7109375"/>
-    <col customWidth="1" min="4" max="4" width="53.00390625"/>
+    <col customWidth="1" min="4" max="4" width="60.00390625"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25">
@@ -743,11 +747,12 @@
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>5</v>
-      </c>
+      <c r="B2" s="3"/>
       <c r="C2" s="4">
         <v>25.629999999999999</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="3" ht="14.25">
@@ -755,10 +760,10 @@
         <v>6</v>
       </c>
       <c r="B3" s="3"/>
-      <c r="C3" s="5">
+      <c r="C3" s="6">
         <v>2.4300000000000002</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="7" t="s">
         <v>7</v>
       </c>
     </row>
@@ -772,7 +777,7 @@
       <c r="C4" s="4">
         <v>4.0300000000000002</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="7" t="s">
         <v>10</v>
       </c>
     </row>
@@ -786,7 +791,7 @@
       <c r="C5" s="4">
         <v>2.7200000000000002</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="7" t="s">
         <v>13</v>
       </c>
     </row>
@@ -794,13 +799,13 @@
       <c r="A6" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="8" t="s">
         <v>15</v>
       </c>
       <c r="C6" s="4">
         <v>2.1699999999999999</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="9" t="s">
         <v>16</v>
       </c>
     </row>
@@ -814,7 +819,7 @@
       <c r="C7" s="4">
         <v>4.9000000000000004</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>19</v>
       </c>
     </row>
@@ -828,7 +833,7 @@
       <c r="C8" s="4">
         <v>10.07</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="7" t="s">
         <v>22</v>
       </c>
     </row>
@@ -842,7 +847,7 @@
       <c r="C9" s="4">
         <v>2.5499999999999998</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="7" t="s">
         <v>25</v>
       </c>
     </row>
@@ -856,7 +861,7 @@
       <c r="C10" s="4">
         <v>1.6100000000000001</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="7" t="s">
         <v>28</v>
       </c>
     </row>
@@ -868,7 +873,7 @@
       <c r="C11" s="4">
         <v>1.28</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="7" t="s">
         <v>30</v>
       </c>
     </row>
@@ -880,17 +885,17 @@
       <c r="C12" s="4">
         <v>7</v>
       </c>
-      <c r="D12" s="9"/>
+      <c r="D12" s="10"/>
     </row>
     <row r="13" ht="14.25">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="10"/>
+      <c r="B13" s="11"/>
       <c r="C13" s="4">
         <v>14.529999999999999</v>
       </c>
-      <c r="D13" s="10"/>
+      <c r="D13" s="11"/>
     </row>
     <row r="14" ht="14.25">
       <c r="A14" s="2" t="s">
@@ -900,7 +905,7 @@
       <c r="C14" s="4">
         <v>12.4</v>
       </c>
-      <c r="D14" s="9"/>
+      <c r="D14" s="10"/>
     </row>
     <row r="15" ht="14.25">
       <c r="A15" s="2" t="s">
@@ -908,37 +913,47 @@
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="4">
-        <v>48.049999999999997</v>
-      </c>
-      <c r="D15" s="9"/>
+        <v>59.950000000000003</v>
+      </c>
+      <c r="D15" s="10"/>
     </row>
     <row r="16" ht="14.25">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="B16" s="10"/>
+      <c r="B16" s="11"/>
       <c r="C16" s="4">
-        <v>44.700000000000003</v>
-      </c>
-      <c r="D16" s="10"/>
+        <v>16.170000000000002</v>
+      </c>
+      <c r="D16" s="11"/>
     </row>
     <row r="17" ht="14.25">
-      <c r="A17" t="s">
+      <c r="A17" s="11" t="s">
         <v>36</v>
       </c>
+      <c r="B17" s="11"/>
       <c r="C17" s="4">
+        <v>17.07</v>
+      </c>
+      <c r="D17" s="11"/>
+    </row>
+    <row r="18" ht="14.25">
+      <c r="A18" t="s">
+        <v>37</v>
+      </c>
+      <c r="C18" s="4">
         <v>14.800000000000001</v>
       </c>
-      <c r="D17" s="9"/>
-    </row>
-    <row r="18" ht="14.25">
-      <c r="A18" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="B18" s="2"/>
-      <c r="C18" s="12">
-        <f>CEILING(SUM(C2:C17),1)</f>
-        <v>199</v>
+      <c r="D18" s="10"/>
+    </row>
+    <row r="19" ht="14.25">
+      <c r="A19" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" s="2"/>
+      <c r="C19" s="13">
+        <f>CEILING(SUM(C2:C18),1)</f>
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>